<commit_message>
remove duplicate datasets/update cleanup files
</commit_message>
<xml_diff>
--- a/05 dependency and cleanup reports/scuc_dependency_scan_and_cleanup_plan.xlsx
+++ b/05 dependency and cleanup reports/scuc_dependency_scan_and_cleanup_plan.xlsx
@@ -1407,7 +1407,7 @@
         <v>40</v>
       </c>
       <c r="E5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" t="b">
         <v>0</v>
@@ -1475,7 +1475,7 @@
         <v>40</v>
       </c>
       <c r="E6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" t="b">
         <v>0</v>
@@ -1543,7 +1543,7 @@
         <v>40</v>
       </c>
       <c r="E7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" t="b">
         <v>0</v>
@@ -1611,7 +1611,7 @@
         <v>40</v>
       </c>
       <c r="E8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" t="b">
         <v>0</v>
@@ -1679,7 +1679,7 @@
         <v>40</v>
       </c>
       <c r="E9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9" t="b">
         <v>0</v>
@@ -1747,7 +1747,7 @@
         <v>40</v>
       </c>
       <c r="E10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" t="b">
         <v>0</v>
@@ -1815,7 +1815,7 @@
         <v>40</v>
       </c>
       <c r="E11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F11" t="b">
         <v>0</v>
@@ -1883,7 +1883,7 @@
         <v>40</v>
       </c>
       <c r="E12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12" t="b">
         <v>0</v>
@@ -1951,7 +1951,7 @@
         <v>40</v>
       </c>
       <c r="E13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" t="b">
         <v>0</v>
@@ -2019,7 +2019,7 @@
         <v>40</v>
       </c>
       <c r="E14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14" t="b">
         <v>0</v>
@@ -2155,7 +2155,7 @@
         <v>85</v>
       </c>
       <c r="E16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16" t="b">
         <v>0</v>
@@ -2223,7 +2223,7 @@
         <v>89</v>
       </c>
       <c r="E17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17" t="b">
         <v>0</v>
@@ -2291,7 +2291,7 @@
         <v>40</v>
       </c>
       <c r="E18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F18" t="b">
         <v>0</v>
@@ -2359,7 +2359,7 @@
         <v>96</v>
       </c>
       <c r="E19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F19" t="b">
         <v>0</v>
@@ -2427,7 +2427,7 @@
         <v>85</v>
       </c>
       <c r="E20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F20" t="b">
         <v>0</v>
@@ -2559,7 +2559,7 @@
         <v>89</v>
       </c>
       <c r="E22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F22" t="b">
         <v>0</v>
@@ -2625,7 +2625,7 @@
         <v>40</v>
       </c>
       <c r="E23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F23" t="b">
         <v>0</v>
@@ -2691,7 +2691,7 @@
         <v>25</v>
       </c>
       <c r="E24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F24" t="b">
         <v>0</v>
@@ -2757,7 +2757,7 @@
         <v>25</v>
       </c>
       <c r="E25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F25" t="b">
         <v>0</v>
@@ -2823,7 +2823,7 @@
         <v>25</v>
       </c>
       <c r="E26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F26" t="b">
         <v>0</v>
@@ -2955,7 +2955,7 @@
         <v>25</v>
       </c>
       <c r="E28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F28" t="b">
         <v>0</v>
@@ -3021,7 +3021,7 @@
         <v>25</v>
       </c>
       <c r="E29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F29" t="b">
         <v>0</v>
@@ -3087,7 +3087,7 @@
         <v>25</v>
       </c>
       <c r="E30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F30" t="b">
         <v>0</v>
@@ -3153,7 +3153,7 @@
         <v>25</v>
       </c>
       <c r="E31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F31" t="b">
         <v>0</v>
@@ -3222,7 +3222,7 @@
         <v>1</v>
       </c>
       <c r="F32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" t="s">
         <v>134</v>
@@ -3256,10 +3256,10 @@
         <v>0</v>
       </c>
       <c r="R32" t="s">
-        <v>101</v>
+        <v>27</v>
       </c>
       <c r="S32" t="s">
-        <v>102</v>
+        <v>28</v>
       </c>
       <c r="T32" t="b">
         <v>0</v>
@@ -3285,7 +3285,7 @@
         <v>137</v>
       </c>
       <c r="E33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F33" t="b">
         <v>0</v>
@@ -3351,7 +3351,7 @@
         <v>96</v>
       </c>
       <c r="E34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F34" t="b">
         <v>0</v>
@@ -3417,7 +3417,7 @@
         <v>96</v>
       </c>
       <c r="E35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F35" t="b">
         <v>0</v>
@@ -3483,7 +3483,7 @@
         <v>96</v>
       </c>
       <c r="E36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F36" t="b">
         <v>0</v>
@@ -3549,7 +3549,7 @@
         <v>96</v>
       </c>
       <c r="E37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F37" t="b">
         <v>0</v>
@@ -3615,7 +3615,7 @@
         <v>96</v>
       </c>
       <c r="E38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F38" t="b">
         <v>0</v>
@@ -3681,7 +3681,7 @@
         <v>96</v>
       </c>
       <c r="E39" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F39" t="b">
         <v>0</v>
@@ -3747,7 +3747,7 @@
         <v>35</v>
       </c>
       <c r="E40" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F40" t="b">
         <v>0</v>

</xml_diff>